<commit_message>
aggiunti url per lo scraping per tripadvisor e aggiunto campo room_type su recensioni booking per calcolare la media per camera
</commit_message>
<xml_diff>
--- a/datasets/general_data_dataset_booking.xlsx
+++ b/datasets/general_data_dataset_booking.xlsx
@@ -526,62 +526,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Camping Village Mar y Sierra</t>
+          <t>Camping La Pineta</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Strada San Gervasio 3, 61039 San Costanzo, Italia</t>
+          <t>Via della repubblica 3, 62017 Porto Recanati, Italia</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>Situato a San Costanzo, il Camping Village Mar y Sierra vanta una piscina all'aperto, la connessione WiFi gratuita nelle aree comuni e camere climatizzate, in alcuni casi con terrazza.
-Ciascuna sistemazione presenta anche una TV a schermo piatto, una scrivania e un bagno privato con set di cortesia.
-Il campeggio comprende anche un campo da tennis, servizi per riunioni, un salone comune e uno staff dedicato per l'intrattenimento.
-Completo di parcheggio gratuito, il Camping Village Mar y Sierra dista, in auto, 10 minuti dalle spiagge della zona e 40 minuti da Pesaro.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>No camping host description</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BAGNO: Carta igienica, Vasca o doccia, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Armadio o guardaroba, | VISTA: Vista giardino, | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Terrazza solarium, Barbecue, Terrazza, Giardino, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ANIMALI: | ATTIVITÀ: Trasmissione di eventi sportivi in diretta, Spettacolo/musica dal vivo, Spiaggia, Armadietti per fitness/spa, Attrezzatura da tennis, Parco acquatico
-Non sul posto
-a pagamento, Intrattenimento serale, Ping-pong, Area giochi, Sala giochi, Campo da tennis, | AREA SOGGIORNO: Zona soggiorno, | SERVIZI DI RISTORAZIONE: Caffetteria sul posto, Vino/champagne
-a pagamento, Pasti per bambini, Menù per diete particolari (su richiesta), Bar, Ristorante, | INTERNET: | PARCHEGGIO: Parcheggio per disabili, Parcheggio in strada, | ALTRI SERVIZI: Sala comune/zona TV, Servizio concierge, Deposito bagagli, Banco escursioni, Spazi per riunioni/banchetti
-a pagamento, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, Area giochi al coperto, | PROTEZIONE E SICUREZZA: Estintori, Telecamere a circuito chiuso all'esterno della struttura, Telecamere a circuito chiuso nelle zone in comune, Allarme antifumo, Allarme di sicurezza, Sicurezza 24 ore su 24, | SERVIZI GENERALI: Aria condizionata, Struttura interamente non fumatori, Riscaldamento, Ingresso indipendente, Disponibilità di camere familiari, Camere/strutture per ospiti disabili, Camere non fumatori, | ACCESSIBILITÀ: Intera unità situata al piano terra, | PISCINA SCOPERTA: Stagionale, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, Scivolo d'acqua, | LINGUE PARLATE: Tedesco, Inglese, Italiano, Olandese, | </t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>camping-village-mar-y-sierra</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Camping La Pineta</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Via della repubblica 3, 62017 Porto Recanati, Italia</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
         <is>
           <t>Situato nella località marchigiana di Porto Recanati, a 25 km da Ancona e a 49 km da Senigallia, il Camping La Pineta vanta un'area giochi per bambini, una spiaggia privata e servizi gratuiti quali la connessione WiFi e un parcheggio privato in loco.
 Alcune sistemazioni dispongono di aria condizionata, di zona pranzo e/o di patio, e su richiesta potrete usufruire di una TV. Avrete a disposizione anche un angolo cottura con frigorifero e fornelli e un bagno privato con vasca o doccia e bidè.
@@ -589,12 +542,12 @@
 Presso la struttura potrete giocare a ping pong e noleggiare biciclette. Il Camping La Pineta dista 13 km da Civitanova Marche e 33 km dall'Aeroporto di Ancona Falconara, il più vicino alla struttura.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Situato in posizione peculiare direttamente sul mare il Camping Pineta offre al proprio ospite un soggiorno di relax e divertimento. A sud di Porto Recanati, a solo 800 mt dal centro del paese, facilmente raggiungibile tramite  una passeggiata pedonale. A pochi passi dalla rinomata Riviera del Conero e da zone di interesse culturale come Loreto e Recanati. All'interno si potra' trovare bar, ristorante, pizzeria, minimarket, noleggio bici, navetta per il centro e animazione serale e diurna dal 01/07. Cani di piccola taglia ammessi</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t xml:space="preserve">BAGNO: Bidet, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Armadio o guardaroba, | VISTA: Vista giardino, | CUCINA: Tavolo da pranzo, Piano cottura, Utensili da cucina, Cucina, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ANIMALI: | ATTIVITÀ: Trasmissione di eventi sportivi in diretta, Spettacolo/musica dal vivo, Tour o lezioni sulla cultura locale
 a pagamento, Happy hour
@@ -609,32 +562,32 @@
 a pagamento, | LINGUE PARLATE: Tedesco, Inglese, Italiano, | </t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>https://www.booking.com/hotel/it/camping-la-pineta.it.html</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>camping-la-pineta</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Saecula Natural Village Experience</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Contrada Ripacorvara, 1, 63086 Force, Italia</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Hai diritto a uno sconto Genius su Saecula Natural Village Experience! Per risparmiare su questa struttura ti basta accedere.
 Situato a Force, il Saecula Natural Village Experience offre la connessione WiFi gratuita e suite dotate di cucina, area salotto e TV a schermo piatto.
@@ -644,7 +597,7 @@
 San Benedetto. La struttura dista 46 km da Del Tronto e 25 km da Ascoli Piceno. L'Aeroporto più vicino è quello di Ancona Falconara, a 116 km da Saecula Natural Village Experience.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>L'Agriturismo, (nuovo) attivo dal 2018,  è composto da:
 -ALLOGGI - (Appartamenti)
@@ -659,7 +612,7 @@
 - tende + stuoie + sacco a pelo.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t xml:space="preserve">BAGNO: Carta igienica, Asciugamani, Bidet, Servizi igienici aggiuntivi, Vasca o doccia, Prodotti da bagno in omaggio, Asciugacapelli, | VISTA: Vista cortile interno, Vista luogo di interesse, Vista montagna, Vista giardino, | SPAZI ALL'APERTO: Camino all'aperto, Area picnic, Arredamento da esterni, Zona pranzo all'aperto, Arredamento da esterno, Terrazza solarium, Barbecue, Barbecue, Terrazza, Giardino, | CUCINA: Prodotti per le pulizie, Lavatrice, | ANIMALI: | ATTIVITÀ: Tour in bicicletta, Tour a piedi, Mostre d'arte temporanee
 Non sul posto, Fitness, Vasca all'aperto, Escursioni in bicicletta, Escursionismo, Ping-pong, Solarium, Palestra, | INTERNET: | PARCHEGGIO: Parcheggio per disabili, Parcheggio in strada, | ALTRI SERVIZI: Armadietti, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, Check-in e check-out privati, Sportello bancomat, Deposito bagagli, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, Giochi da tavolo/puzzle, Libri, DVD o musica per bambini, Giochi da tavolo/puzzle, Copriprese di sicurezza per bambini, | SERVIZI DI PULIZIA: Servizio pulizie giornaliero
@@ -667,14 +620,63 @@
 a pagamento, | PROTEZIONE E SICUREZZA: Estintori, Accesso con chiavi, | SERVIZI GENERALI: Ciotole per animali domestici, Ceste per animali domestici, Minimarket sul posto, Area fumatori, Aria condizionata, Camera anallergica, Riscaldamento, Possibilità di pranzo al sacco, Cappella o luogo di culto, Disponibilità di camere insonorizzate, Disponibilità di camere familiari, Parrucchiere/salone di bellezza, Camere/strutture per ospiti disabili, Camere non fumatori, | ACCESSIBILITÀ: Campanello di emergenza nel bagno, Lavabo più basso, WC con seduta più alta, WC con maniglioni, Accesso su sedia a rotelle, | SERVIZI BENESSERE: Sdraio/lettini, Teli da piscina/spiaggia, | LINGUE PARLATE: Inglese, Francese, Italiano, | </t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/saecula.it.html</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>saecula</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fattoria country village</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>contrada fonte san giovanni 3 montecarotto contrada fonte san giovanni 3, 60036 Montecarotto, Italia</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Hai diritto a uno sconto Genius su fattoria country village! Per risparmiare su questa struttura ti basta accedere.
+Situato a Montecarotto, nelle Marche, il Fattoria Country Village offre sistemazioni con parcheggio privato gratuito.
+A disposizione un bagno in comune completamente attrezzato con bidet e set di cortesia.
+Al mattino vi attende una colazione a buffet o all'italiana.
+Potrete approfittare di un barbecue e rilassarvi in giardino o nell’area salotto in comune.
+Il Fattoria Country Village dista 45 km da Sirolo e 26 km da Senigallia. A 39 km raggiungerete l’Aeroporto di Ancona-Falconara, lo scalo più vicino.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No camping host description</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCHEGGIO: Parcheggio custodito, | INTERNET: | CUCINA: Cucina in comune, | BAGNO: Carta igienica, Bidet, Vasca o doccia, Servizi igienici in comune, WC, Prodotti da bagno in omaggio, Bagno in comune, Vasca, Doccia, | AREA SOGGIORNO: Zona soggiorno, | SERVIZI IN CAMERA: Stendibiancheria, | ANIMALI: | ACCESSIBILITÀ: Campanello di emergenza nel bagno, Lavabo più basso, WC con seduta più alta, WC con maniglioni, Accesso su sedia a rotelle, | SPAZI ALL'APERTO: Camino all'aperto, Area picnic, Barbecue, Barbecue, Giardino, | PISCINA SCOPERTA: Stagionale, Orari di apertura, Accessibile a ogni età, Teli da piscina/spiaggia, Sdraio/lettini, Giochi da piscina, Ombrelloni, Piscina con vista, | SERVIZI BENESSERE: Sdraio/lettini, Teli da piscina/spiaggia, | SERVIZI GENERALI: Ciotole per animali domestici, WiFi a pagamento, Sala comune/zona TV, Servizio navetta (a pagamento), Possibilità di pranzo al sacco, Cappella o luogo di culto, Camere/strutture per ospiti disabili, Cassaforte, | SERVIZI DI RISTORAZIONE: Caffetteria sul posto, Vino/champagne
+a pagamento, Pasti per bambini, Snack bar, | ATTIVITÀ: Tiro con l'arco, Happy hour
+a pagamento, Tour in bicicletta, Tour a piedi
+a pagamento, Giro dei pub
+a pagamento, Attrezzatura da badminton, Vasca all'aperto, Staff di animazione, Escursioni in bicicletta, Ping-pong, Pesca, | VISTA: Vista, | SERVIZI DI ACCOGLIENZA: Check-in e check-out privati, Reception 24 ore su 24, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, Area giochi al coperto, Giochi da tavolo/puzzle, | SERVIZI BUSINESS: Fax/fotocopiatrice, | LINGUE PARLATE: Inglese, Spagnolo, | </t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html</t>
+          <t>https://www.booking.com/hotel/it/fattoria-country-village.it.html</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>fattoria-country-village</t>
         </is>
       </c>
     </row>
@@ -684,58 +686,15 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>La Bolla del Borgo. Le Marche tra le stelle.</t>
+          <t>Camping Led Zeppelin</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Via Olmigrandi 72, 60013 Corinaldo, Italia</t>
+          <t>5 Contrada Boccabianca, 63064 Cupra Marittima, Italia</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
-        <is>
-          <t>Situato a Corinaldo, nelle Marche, il campeggio La Bolla del Borgo. Le Marche tra le stelle. offre un giardino. Dotata di un parcheggio privato gratuito, la struttura si trova a 37 km da Ancona.
-Potrete usufruire di lenzuola e asciugamani.
-Il campeggio serve una colazione all'italiana o senza glutine.
-Il Bolla del Borgo. Le Marche tra le stelle. dista 49 km da Riccione e 48 km da Sirolo. L’Aeroporto di Ancona-Falconara è lo scalo più vicino e sorge a 24 km.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>No camping host description</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | CAMERA DA LETTO: Biancheria per la casa, | BAGNO: Carta igienica, Asciugamani, Doccia, | SPAZI ALL'APERTO: Arredamento da esterno, Giardino, | SERVIZI GENERALI: Camere non fumatori, | ALTRI SERVIZI: Check-in e check-out privati, Check-in e check-out express, | VISTA: Vista, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | LINGUE PARLATE: Inglese, Francese, Italiano, Giapponese, | </t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/la-bolla-del-borgo-le-marche-tra-le-stelle-provincia-di-ancona.it.html</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>la-bolla-del-borgo-le-marche-tra-le-stelle-provincia-di-ancona</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Camping Led Zeppelin</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>5 Contrada Boccabianca, 63064 Cupra Marittima, Italia</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
         <is>
           <t>Questa struttura si trova a 1 minuto a piedi dalla spiaggia. Situato a Cupra Marittima, il Camping Led Zeppelin offre una vista sul proprio giardino, un ristorante, il servizio in camera, un bar, una piscina all’aperto stagionale e un’area giochi per bambini.
 Gli alloggi dispongono di aria condizionata, terrazza, TV a schermo piatto e bagno privato con doccia e set di cortesia. Alcune sistemazioni includono una cucina con microonde e piano cottura.
@@ -743,12 +702,12 @@
 Il Camping Led Zeppelin dista 10 km da San Benedetto del Tronto e 46 km da Porto Recanati. L’Aeroporto d’Abruzzo, lo scalo più vicino, è ubicato a 73 km.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>No camping host description</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t xml:space="preserve">BAGNO: Carta igienica, Asciugamani, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Prodotti da bagno in omaggio, Doccia, | VISTA: Vista giardino, | SPAZI ALL'APERTO: Arredamento da esterno, Terrazza, Giardino, | CUCINA: Frigorifero, | ANIMALI: | ATTIVITÀ: Trasmissione di eventi sportivi in diretta, Spettacolo/musica dal vivo, Serate di cinema, Cabaret, Spiaggia, Lezioni di fitness, Intrattenimento serale, Fronte spiaggia, Mini club, Locale notturno/DJ, Staff di animazione, Spiaggia privata
 a pagamento, Karaoke, Area giochi, Pesca, Campo da tennis
@@ -757,14 +716,57 @@
 a pagamento, | ALTRI SERVIZI: Servizio lavanderia, Servizio in camera, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, Area giochi al coperto, Giochi da tavolo/puzzle, | PROTEZIONE E SICUREZZA: Estintori, Telecamere a circuito chiuso nelle zone in comune, Allarme antifumo, Allarme di sicurezza, Sicurezza 24 ore su 24, | SERVIZI GENERALI: WiFi a pagamento, Minimarket sul posto, Aria condizionata, Struttura interamente non fumatori, Riscaldamento, Ingresso indipendente, Ascensore, Disponibilità di camere familiari, | ACCESSIBILITÀ: Intera unità situata al piano terra, | PISCINA SCOPERTA: Stagionale, Accessibile a ogni età, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | LINGUE PARLATE: Inglese, Italiano, | </t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/camping-led-zeppelin.it.html</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>camping-led-zeppelin</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>La Bolla del Borgo. Le Marche tra le stelle.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Via Olmigrandi 72, 60013 Corinaldo, Italia</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Situato a Corinaldo, nelle Marche, il campeggio La Bolla del Borgo. Le Marche tra le stelle. offre un giardino. Dotata di un parcheggio privato gratuito, la struttura si trova a 37 km da Ancona.
+Potrete usufruire di lenzuola e asciugamani.
+Il campeggio serve una colazione all'italiana o senza glutine.
+Il Bolla del Borgo. Le Marche tra le stelle. dista 49 km da Riccione e 48 km da Sirolo. L’Aeroporto di Ancona-Falconara è lo scalo più vicino e sorge a 24 km.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No camping host description</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | CAMERA DA LETTO: Biancheria per la casa, | BAGNO: Carta igienica, Asciugamani, Doccia, | SPAZI ALL'APERTO: Arredamento da esterno, Giardino, | SERVIZI GENERALI: Camere non fumatori, | ALTRI SERVIZI: Check-in e check-out privati, Check-in e check-out express, | VISTA: Vista, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | LINGUE PARLATE: Inglese, Francese, Italiano, Giapponese, | </t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-led-zeppelin.it.html</t>
+          <t>https://www.booking.com/hotel/it/la-bolla-del-borgo-le-marche-tra-le-stelle-provincia-di-ancona.it.html</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>camping-led-zeppelin</t>
+          <t>la-bolla-del-borgo-le-marche-tra-le-stelle-provincia-di-ancona</t>
         </is>
       </c>
     </row>
@@ -915,40 +917,44 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Resort Orizzonti Glamping</t>
+          <t>Camping Village Mar y Sierra</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1081 Via Monte Taccone, 63811 Sant'Elpidio a Mare, Italia</t>
+          <t>Strada San Gervasio 3, 61039 San Costanzo, Italia</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Set in SantʼElpidio a Mare, Resort Orizzonti Glamping offers accommodation with air conditioning and access to a garden with an outdoor swimming pool.
-There is a fully equipped private bathroom with shower and a hairdryer.
-The tented camp provides a barbecue.
-San Benedetto del Tronto is 36 km from Resort Orizzonti Glamping, while Sirolo is 31 km away. The nearest airport is Ancona Falconara Airport, 48 km from the accommodation.</t>
+          <t>Situato a San Costanzo, il Camping Village Mar y Sierra vanta una piscina all'aperto, la connessione WiFi gratuita nelle aree comuni e camere climatizzate, in alcuni casi con terrazza.
+Ciascuna sistemazione presenta anche una TV a schermo piatto, una scrivania e un bagno privato con set di cortesia.
+Il campeggio comprende anche un campo da tennis, servizi per riunioni, un salone comune e uno staff dedicato per l'intrattenimento.
+Completo di parcheggio gratuito, il Camping Village Mar y Sierra dista, in auto, 10 minuti dalle spiagge della zona e 40 minuti da Pesaro.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>La collocazione sopraelevata garantisce un'incantevole vista sulle colline marchigiane e sugli spazi verdi della Riserva naturale, all'orizzonte  scorgono </t>
+          <t>No camping host description</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAGNO: Carta igienica, Asciugamani, Bagno privato, WC, Asciugacapelli, Doccia, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | VISTA: Vista giardino, | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Zona pranzo all'aperto, Arredamento da esterno, Barbecue, Barbecue, Giardino, | CUCINA: Cucina in comune, Tavolo da pranzo, Utensili da cucina, Frigorifero, | SERVIZI IN CAMERA: Stand appendiabiti, | ANIMALI: | AREA SOGGIORNO: Zona pranzo, Zona soggiorno, | INTERNET: | PARCHEGGIO: | ALTRI SERVIZI: Possibilità di pranzo al sacco, Servizio lavanderia, | SERVIZI GENERALI: Area fumatori, Aria condizionata, Struttura interamente non fumatori, Riscaldamento, Disponibilità di camere familiari, Camere non fumatori, | PISCINA SCOPERTA: Stagionale, Accessibile a ogni età, Piscina con vista, Zona acqua bassa, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | LINGUE PARLATE: Italiano, | </t>
+          <t xml:space="preserve">BAGNO: Carta igienica, Vasca o doccia, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Armadio o guardaroba, | VISTA: Vista giardino, | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Terrazza solarium, Barbecue, Terrazza, Giardino, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ANIMALI: | ATTIVITÀ: Trasmissione di eventi sportivi in diretta, Spettacolo/musica dal vivo, Spiaggia, Armadietti per fitness/spa, Attrezzatura da tennis, Parco acquatico
+Non sul posto
+a pagamento, Intrattenimento serale, Ping-pong, Area giochi, Sala giochi, Campo da tennis, | AREA SOGGIORNO: Zona soggiorno, | SERVIZI DI RISTORAZIONE: Caffetteria sul posto, Vino/champagne
+a pagamento, Pasti per bambini, Menù per diete particolari (su richiesta), Bar, Ristorante, | INTERNET: | PARCHEGGIO: Parcheggio per disabili, Parcheggio in strada, | ALTRI SERVIZI: Sala comune/zona TV, Servizio concierge, Deposito bagagli, Banco escursioni, Spazi per riunioni/banchetti
+a pagamento, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, Area giochi al coperto, | PROTEZIONE E SICUREZZA: Estintori, Telecamere a circuito chiuso all'esterno della struttura, Telecamere a circuito chiuso nelle zone in comune, Allarme antifumo, Allarme di sicurezza, Sicurezza 24 ore su 24, | SERVIZI GENERALI: Aria condizionata, Struttura interamente non fumatori, Riscaldamento, Ingresso indipendente, Disponibilità di camere familiari, Camere/strutture per ospiti disabili, Camere non fumatori, | ACCESSIBILITÀ: Intera unità situata al piano terra, | PISCINA SCOPERTA: Stagionale, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, Scivolo d'acqua, | LINGUE PARLATE: Tedesco, Inglese, Italiano, Olandese, | </t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/resort-orizzonti-glamping.it.html</t>
+          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>resort-orizzonti-glamping</t>
+          <t>camping-village-mar-y-sierra</t>
         </is>
       </c>
     </row>
@@ -958,156 +964,15 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Agricampeggio Abbruzzetti</t>
+          <t>Lodge Holidays - Camping Podere Sei Poorte</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Via San Pietro Vecchio, 63900 Marina Palmense, Italia</t>
+          <t>Via Petricci, 61020 Genga, Italia</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
-        <is>
-          <t>Situato a Marina Palmense, l'Agricampeggio Abbruzzetti offre una piscina, un ristorante, un giardino, una vista sulla piscina e la connessione WiFi gratuita.
-Le sistemazioni presentano un patio affacciato sul giardino, una cucina con forno a microonde e frigorifero, e un bagno privato con bidet. Al loro interno troverete un’area salotto e una zona pranzo.
-Il campeggio mette a vostra disposizione un barbecue.
-L'Agricampeggio Abbruzzetti dista 1,7 km dalla spiaggia di Porto San Giorgio e 70 km dall’Aeroporto di Ancona-Falconara, lo scalo più vicino.</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No camping host description</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BAGNO: Bidet, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Doccia, | VISTA: Vista luogo di interesse, Vista montagna, Vista piscina, Vista giardino, Vista mare, | SPAZI ALL'APERTO: Area picnic, Zona pranzo all'aperto, Barbecue, Barbecue, Patio, Giardino, | CUCINA: Tavolo da pranzo, Piano cottura, Utensili da cucina, Cucina, Forno a microonde, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Stendibiancheria, Stand appendiabiti, | ANIMALI: | AREA SOGGIORNO: Zona pranzo, Zona soggiorno, | SERVIZI DI RISTORAZIONE: Pasti per bambini
-a pagamento, Ristorante, | INTERNET: | PARCHEGGIO: Parcheggio custodito, | ALTRI SERVIZI: Possibilità di pranzo al sacco, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | PROTEZIONE E SICUREZZA: Estintori, | SERVIZI GENERALI: Struttura interamente non fumatori, Zanzariera, Pavimento in marmo o in piastrelle, Ingresso indipendente, Riscaldamento, | PISCINA SCOPERTA: Stagionale, Accessibile a ogni età, Recinto attorno alla piscina, Sdraio/lettini, Ombrelloni, Piscina a sfioro, Piscina con vista, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | LINGUE PARLATE: Inglese, Italiano, | </t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/agricampeggio-abbruzzetti.it.html</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>agricampeggio-abbruzzetti</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Antica Dimora - GLAMPING FIORDALISO</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>C.DA CALLARELLA, 62028 Sarnano, Italia</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Situata a Sarnano, nelle Marche, l'ANTICA DIMORA - CAMPEGGIO FIORDALISO offre gratuitamente il WiFi e un parcheggio privato.
-Potrete nuotare nella piscina all'aperto, sciare o andare in bicicletta, o rilassarvi nel giardino e utilizzare il barbecue.
-Il campeggio dista 48 km da Grottammare e 44 km da Porto San Giorgio. L'ANTICA DIMORA - CAMPEGGIO FIORDALISO dista 63 km dall'Aeroporto di Ancona Falconara, lo scalo più vicino.</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Il campeggio Fiordaliso è stato pensato per offrire agli ospiti un ambiente naturale e verde, con una bella vista sui Monti Sibillini  godendo di tutti i nuovissimi servizi appena allestiti e di una bella piscina. E' un campeggio per tende e roulotte.
-Abbiamo voluto creare un ambiente per "volare al di fuori del tempo", nei luoghi magici e fantastici di " Alice nel Paese delle Meraviglie".
-Potrete alloggiare in delle bellissime roulotte rivisitate dove incontrerete lo Stregatto o il  Bianconiglio o piuttosto il Cappellaio Magico perchè la nostra parola d'ordine è MERAVIGLIARSI SEMPRE....meravigliarsi delle lucciole che ci fanno luce nelle sere di giugno , delle stelle così brillanti che sembra di toccare con la mano, dei concerti al chiaro di luna intonati dalle nostre rane, dalla tenerezza di tutti i nostri amici della fattoria che ci fanno da cornice. 
-C'è un posto che non ha eguali sulla terra....Questo luogo è un luogo unico al mondo, una terra colma di meraviglie, mistero e pericolo. Si dice che per sopravvivere qui bisogna essere matti come un cappellaio. E per fortuna...io lo sono. "</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | BAGNO: Bagno in comune, | SPAZI ALL'APERTO: Area picnic, Barbecue, Giardino, | PISCINA SCOPERTA: Stagionale, Sdraio/lettini, Piscina con vista, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | SERVIZI GENERALI: Disponibilità di camere familiari, Camere non fumatori, | ATTIVITÀ: Tour in bicicletta
-a pagamento, Tour a piedi, Escursioni in bicicletta
-Non sul posto, Escursionismo
-Non sul posto, Noleggio biciclette (a pagamento), Sci, | ALTRI SERVIZI: Check-in e check-out express, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | PROTEZIONE E SICUREZZA: Accesso con chiavi, | LINGUE PARLATE: Inglese, Italiano, | </t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/antica-dimora-campeggio-fiordaliso.it.html</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>antica-dimora-campeggio-fiordaliso</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Camping Blu Fantasy</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Lungomare Italia 3B, 60019 Senigallia, Italia</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Situato sul lungomare, a 4 km da Senigallia, il Camping Blu Fantasy offre appartamenti a ristorazione indipendente, una piscina all’aperto e un giardino con barbecue. Il WiFi è fruibile gratuitamente nelle aree comuni.
-Tutti gli appartamenti sono dotati di aria condizionata, TV a schermo piatto e angolo cottura con forno e frigorifero. Presentano anche un bagno privato con doccia e bidè.
-I più piccoli apprezzeranno il programma di intrattenimento e l’area giochi a loro dedicati. Tra i servizi troverete inoltre un bar, un minimarket e un ristorante esterno convenzionato con trattamento di mezza pensione e pensione completa.
-Il Camping Villaggio Blu si trova a 15 minuti d’auto da Falconara Marittima e a 30 km da Jesi.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>La data di apertura del Villaggio è prevista dal 1° giugno all'11 settembre 2022 compreso, con tutti i servizi operativi, nel rispetto delle norme governative sulla sicurezza e la salute dei nostri ospiti. 
-La biancheria NON è inclusa nel prezzo del soggiorno. Il kit di biancheria completo da letto e da bagno è valido per l'intero soggiorno ed è da noleggiare su richiesta al momento della prenotazione del soggiorno. Il costo per un kit matrimoniale è di 18 Euro, mentre quello del kit singolo di 11,5 Euro. In alternativa si dovrà utilizzare la propria biancheria dal letto e da bagno.
-Il servizio spiaggia NON è incluso nel prezzo del soggiorno. Vi sono 2 stabilimenti balneari con sabbia aggiunta nelle vicinanze; spiaggia convenzionata "TRILLO 148" a 600 metri oppure spiaggia NON convenzionata "Bahya Blanca"a 150 metri (più piccola e meno attrezzata). Spiaggia libera di ghiaia con fondale sabbioso di fronte a noi, a 50 metri.
-Vi aspettiamo!</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BAGNO: Asciugamani/lenzuola disponibili a pagamento, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Armadio o guardaroba, | SPAZI ALL'APERTO: Barbecue, Giardino, | CUCINA: Tavolo da pranzo, Piano cottura, Utensili da cucina, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ATTIVITÀ: Aerobica, Cabaret, Intrattenimento serale, Mini club, Staff di animazione, Vasca idromassaggio/jacuzzi, Freccette, Karaoke, Ping-pong, Area giochi, | AREA SOGGIORNO: Zona pranzo, Zona soggiorno, | MEDIA E TECNOLOGIA: TV a schermo piatto, Canali satellitari, | SERVIZI DI RISTORAZIONE: Frutta
-a pagamento, Vino/champagne
-a pagamento, Buffet per bambini, Pasti per bambini, Menù per diete particolari (su richiesta), Snack bar, Bar, Ristorante, | INTERNET: | PARCHEGGIO: Parcheggio in strada, | ALTRI SERVIZI: Servizio navetta, Sala comune/zona TV, Servizio navetta (gratuito), Possibilità di pranzo al sacco, Servizio lavanderia
-a pagamento, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Cancelletti di sicurezza per bambini, Area giochi all'aperto, | PROTEZIONE E SICUREZZA: Estintori, Telecamere a circuito chiuso nelle zone in comune, Accesso con chiavi, | SERVIZI GENERALI: Minimarket sul posto, Aria condizionata, Struttura interamente non fumatori, Zanzariera, Riscaldamento, Ingresso indipendente, Disponibilità di camere familiari, Camere non fumatori, | 2 PISCINE: Stagionale, Recinto attorno alla piscina, Sdraio/lettini, Zona acqua bassa, Anche per bambini, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | LINGUE PARLATE: Inglese, Francese, Italiano, | </t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/villaggio-camping-blu.it.html</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>villaggio-camping-blu</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Lodge Holidays - Camping Podere Sei Poorte</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Via Petricci, 61020 Genga, Italia</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
         <is>
           <t>Lodge Holidays - Camping. Situato a Genga, il Podere Sei Poorte offre un ristorante, una piscina all'aperto e un bar. 38 km da Cattolica.
 L'alloggio presenta un'area salotto e un angolo cottura con frigorifero e fornelli.
@@ -1115,7 +980,7 @@
 Il Camping Podere Sei Poorte dista 45 km da Riccione e 23 km da Pesaro. La struttura dista 30 km dall'Aeroporto Internazionale Federico Fellini, lo scalo più vicino.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>If enjoying your holiday might mean more to you than just laying in the sun and could be a combination of just relaxing, cultural development, natural challenges and Italian gastronimical hospitality…………… than Campsite Podere Sei Poorte is your ideal destination. 
 This is truly a fabulous place to spend a holiday and enjoy all the beautiful things life has to offer. The restaurant conjures up delicious pure Italian dishes, à la carte, as well as themed evenings with a pizza buffet, fresh fish, or pasta e basta. 
@@ -1125,19 +990,157 @@
 Laze in the perfectly appointed Fatboy hammock with panoramic views from your luxury Lodge Holidays lodge.</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCHEGGIO: Stazione di ricarica per veicoli elettrici, Parcheggio custodito, | INTERNET: | CUCINA: Seggiolone, Tavolo da pranzo, Piano cottura, Utensili da cucina, Frigorifero, Angolo cottura, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | BAGNO: Carta igienica, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Doccia, | AREA SOGGIORNO: Zona soggiorno, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ANIMALI: | ACCESSIBILITÀ: Intera unità situata al piano terra, | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Zona pranzo all'aperto, Arredamento da esterno, Terrazza solarium, Barbecue, Terrazza, Giardino, | PISCINA SCOPERTA: Aperta tutto l'anno, Sdraio/lettini, Zona acqua bassa, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | SERVIZI GENERALI: Minimarket sul posto, Struttura interamente non fumatori, Ingresso indipendente, Riscaldamento, Disponibilità di camere familiari, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Snack bar, Bar, Ristorante, Bollitore tè/macchina caffè, | ATTIVITÀ: Tour in bicicletta, Tour a piedi, Vasca comune (daiyokujo), Intrattenimento serale, Mini club, Escursioni in bicicletta, Noleggio biciclette (a pagamento), Ping-pong, Area giochi, | ALTRI SERVIZI: Sala comune/zona TV, Check-in e check-out privati, | VISTA: Vista montagna, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, | LINGUE PARLATE: Tedesco, Inglese, Italiano, Olandese, | </t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/camping-podere-sei-poorte.it.html</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>camping-podere-sei-poorte</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Safaritent Glamping Mar Y Sierrra</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>via S. Gervasio, 61039 Casa Castellani, Italia</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Situato a Casa Castellani, il Safaritent Glamping Mar Y Sierrra offre un ristorante, una piscina stagionale all'aperto e un bar. La struttura dista 37 km da Urbino e dispone di un parcheggio privato gratuito.
+In loco troverete anche un'area giochi per bambini. Durante il vostro soggiorno al Safaritent Glamping Mar Y Sierrra potrete giocare a ping pong in loco o esplorare i dintorni in bicicletta.
+La struttura dista 41 km da Ancona e 27 km da Pesaro. Il Safaritent Glamping Mar Y Sierrra dista 25 km dall'Aeroporto di Ancona Falconara, lo scalo più vicino.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No camping host description</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCHEGGIO: Parcheggio per disabili, | INTERNET: | CUCINA: Utensili da cucina, | CAMERA DA LETTO: Biancheria per la casa, | BAGNO: Vasca o doccia, Bagno privato, WC, Doccia, | SPAZI ALL'APERTO: Arredamento da esterni, Arredamento da esterno, Terrazza solarium, Barbecue, Barbecue, Terrazza, Giardino, | PISCINA SCOPERTA: Stagionale, Accessibile a ogni età, Sdraio/lettini, Bar a bordo piscina, Ombrelloni, Scivolo d'acqua, Zona acqua bassa, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, Scivolo d'acqua, | SERVIZI GENERALI: Minimarket sul posto, Struttura interamente non fumatori, Zanzariera, Parquet o pavimento in legno, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Vino/champagne
+a pagamento, Pasti per bambini, Bar, Ristorante, Bollitore tè/macchina caffè, | ATTIVITÀ: Tour in bicicletta, Tour a piedi, Snorkeling
+Non sul posto, Equitazione
+Non sul posto, Escursioni in bicicletta
+Non sul posto, Vasca idromassaggio/jacuzzi, Windsurf
+Non sul posto, Ping-pong, Area giochi, Campo da tennis, | ALTRI SERVIZI: Check-in e check-out privati, | VISTA: Vista montagna, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, | LINGUE PARLATE: Tedesco, Inglese, Italiano, Olandese, | </t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/safaritent-glamping-mar-y-sierrra.it.html</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>safaritent-glamping-mar-y-sierrra</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Antica Dimora - GLAMPING FIORDALISO</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>C.DA CALLARELLA, 62028 Sarnano, Italia</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Situata a Sarnano, nelle Marche, l'ANTICA DIMORA - CAMPEGGIO FIORDALISO offre gratuitamente il WiFi e un parcheggio privato.
+Potrete nuotare nella piscina all'aperto, sciare o andare in bicicletta, o rilassarvi nel giardino e utilizzare il barbecue.
+Il campeggio dista 48 km da Grottammare e 44 km da Porto San Giorgio. L'ANTICA DIMORA - CAMPEGGIO FIORDALISO dista 63 km dall'Aeroporto di Ancona Falconara, lo scalo più vicino.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Il campeggio Fiordaliso è stato pensato per offrire agli ospiti un ambiente naturale e verde, con una bella vista sui Monti Sibillini  godendo di tutti i nuovissimi servizi appena allestiti e di una bella piscina. E' un campeggio per tende e roulotte.
+Abbiamo voluto creare un ambiente per "volare al di fuori del tempo", nei luoghi magici e fantastici di " Alice nel Paese delle Meraviglie".
+Potrete alloggiare in delle bellissime roulotte rivisitate dove incontrerete lo Stregatto o il  Bianconiglio o piuttosto il Cappellaio Magico perchè la nostra parola d'ordine è MERAVIGLIARSI SEMPRE....meravigliarsi delle lucciole che ci fanno luce nelle sere di giugno , delle stelle così brillanti che sembra di toccare con la mano, dei concerti al chiaro di luna intonati dalle nostre rane, dalla tenerezza di tutti i nostri amici della fattoria che ci fanno da cornice. 
+C'è un posto che non ha eguali sulla terra....Questo luogo è un luogo unico al mondo, una terra colma di meraviglie, mistero e pericolo. Si dice che per sopravvivere qui bisogna essere matti come un cappellaio. E per fortuna...io lo sono. "</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | BAGNO: Bagno in comune, | SPAZI ALL'APERTO: Area picnic, Barbecue, Giardino, | PISCINA SCOPERTA: Stagionale, Sdraio/lettini, Piscina con vista, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | SERVIZI GENERALI: Disponibilità di camere familiari, Camere non fumatori, | ATTIVITÀ: Tour in bicicletta
+a pagamento, Tour a piedi, Escursioni in bicicletta
+Non sul posto, Escursionismo
+Non sul posto, Noleggio biciclette (a pagamento), Sci, | ALTRI SERVIZI: Check-in e check-out express, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | PROTEZIONE E SICUREZZA: Accesso con chiavi, | LINGUE PARLATE: Inglese, Italiano, | </t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/antica-dimora-campeggio-fiordaliso.it.html</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>antica-dimora-campeggio-fiordaliso</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Resort Orizzonti Glamping</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1081 Via Monte Taccone, 63811 Sant'Elpidio a Mare, Italia</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Set in SantʼElpidio a Mare, Resort Orizzonti Glamping offers accommodation with air conditioning and access to a garden with an outdoor swimming pool.
+There is a fully equipped private bathroom with shower and a hairdryer.
+The tented camp provides a barbecue.
+San Benedetto del Tronto is 36 km from Resort Orizzonti Glamping, while Sirolo is 31 km away. The nearest airport is Ancona Falconara Airport, 48 km from the accommodation.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>La collocazione sopraelevata garantisce un'incantevole vista sulle colline marchigiane e sugli spazi verdi della Riserva naturale, all'orizzonte  scorgono  i monti Sibillini,  dal  Vettore,alla Sibilla  .Questa vista garantisce riservatezza e tranquillità.Attorno un ampio giardino verde con incantevoli ulivi anche secolari, piscina con vista   e con i suoi 3 appartamenti con ingresso indipendenti 2 tende Glampin di lusso completi di ogni confort, .Rende così  il resort Orizzonti un posto unico e speciale.  Siamo noi tutto lo staff di Resort Orizzonti, a prenderci cura di ogni nostro ospite, che aver così accesso non soltanto a una location di pregio ma a un'esperienza esclusiva .</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARCHEGGIO: Stazione di ricarica per veicoli elettrici, Parcheggio custodito, | INTERNET: | CUCINA: Seggiolone, Tavolo da pranzo, Piano cottura, Utensili da cucina, Frigorifero, Angolo cottura, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | BAGNO: Carta igienica, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Doccia, | AREA SOGGIORNO: Zona soggiorno, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ANIMALI: | ACCESSIBILITÀ: Intera unità situata al piano terra, | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Zona pranzo all'aperto, Arredamento da esterno, Terrazza solarium, Barbecue, Terrazza, Giardino, | PISCINA SCOPERTA: Aperta tutto l'anno, Sdraio/lettini, Zona acqua bassa, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | SERVIZI GENERALI: Minimarket sul posto, Struttura interamente non fumatori, Ingresso indipendente, Riscaldamento, Disponibilità di camere familiari, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Snack bar, Bar, Ristorante, Bollitore tè/macchina caffè, | ATTIVITÀ: Tour in bicicletta, Tour a piedi, Vasca comune (daiyokujo), Intrattenimento serale, Mini club, Escursioni in bicicletta, Noleggio biciclette (a pagamento), Ping-pong, Area giochi, | ALTRI SERVIZI: Sala comune/zona TV, Check-in e check-out privati, | VISTA: Vista montagna, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, | LINGUE PARLATE: Tedesco, Inglese, Italiano, Olandese, | </t>
+          <t xml:space="preserve">BAGNO: Carta igienica, Asciugamani, Bagno privato, WC, Asciugacapelli, Doccia, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | VISTA: Vista giardino, | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Zona pranzo all'aperto, Arredamento da esterno, Barbecue, Barbecue, Giardino, | CUCINA: Cucina in comune, Tavolo da pranzo, Utensili da cucina, Frigorifero, | SERVIZI IN CAMERA: Stand appendiabiti, | ANIMALI: | AREA SOGGIORNO: Zona pranzo, Zona soggiorno, | INTERNET: | PARCHEGGIO: | ALTRI SERVIZI: Possibilità di pranzo al sacco, Servizio lavanderia, | SERVIZI GENERALI: Area fumatori, Aria condizionata, Struttura interamente non fumatori, Riscaldamento, Disponibilità di camere familiari, Camere non fumatori, | PISCINA SCOPERTA: Stagionale, Accessibile a ogni età, Piscina con vista, Zona acqua bassa, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | LINGUE PARLATE: Italiano, | </t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-podere-sei-poorte.it.html</t>
+          <t>https://www.booking.com/hotel/it/resort-orizzonti-glamping.it.html</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>camping-podere-sei-poorte</t>
+          <t>resort-orizzonti-glamping</t>
         </is>
       </c>
     </row>
@@ -1147,15 +1150,64 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>Camping Blu Fantasy</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Lungomare Italia 3B, 60019 Senigallia, Italia</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Situato sul lungomare, a 4 km da Senigallia, il Camping Blu Fantasy offre appartamenti a ristorazione indipendente, una piscina all’aperto e un giardino con barbecue. Il WiFi è fruibile gratuitamente nelle aree comuni.
+Tutti gli appartamenti sono dotati di aria condizionata, TV a schermo piatto e angolo cottura con forno e frigorifero. Presentano anche un bagno privato con doccia e bidè.
+I più piccoli apprezzeranno il programma di intrattenimento e l’area giochi a loro dedicati. Tra i servizi troverete inoltre un bar, un minimarket e un ristorante esterno convenzionato con trattamento di mezza pensione e pensione completa.
+Il Camping Villaggio Blu si trova a 15 minuti d’auto da Falconara Marittima e a 30 km da Jesi.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>La data di apertura del Villaggio è prevista dal 1° giugno all'11 settembre 2022 compreso, con tutti i servizi operativi, nel rispetto delle norme governative sulla sicurezza e la salute dei nostri ospiti. 
+La biancheria NON è inclusa nel prezzo del soggiorno. Il kit di biancheria completo da letto e da bagno è valido per l'intero soggiorno ed è da noleggiare su richiesta al momento della prenotazione del soggiorno. Il costo per un kit matrimoniale è di 18 Euro, mentre quello del kit singolo di 11,5 Euro. In alternativa si dovrà utilizzare la propria biancheria dal letto e da bagno.
+Il servizio spiaggia NON è incluso nel prezzo del soggiorno. Vi sono 2 stabilimenti balneari con sabbia aggiunta nelle vicinanze; spiaggia convenzionata "TRILLO 148" a 600 metri oppure spiaggia NON convenzionata "Bahya Blanca"a 150 metri (più piccola e meno attrezzata). Spiaggia libera di ghiaia con fondale sabbioso di fronte a noi, a 50 metri.
+Vi aspettiamo!</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAGNO: Asciugamani/lenzuola disponibili a pagamento, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Armadio o guardaroba, | SPAZI ALL'APERTO: Barbecue, Giardino, | CUCINA: Tavolo da pranzo, Piano cottura, Utensili da cucina, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ATTIVITÀ: Aerobica, Cabaret, Intrattenimento serale, Mini club, Staff di animazione, Vasca idromassaggio/jacuzzi, Freccette, Karaoke, Ping-pong, Area giochi, | AREA SOGGIORNO: Zona pranzo, Zona soggiorno, | MEDIA E TECNOLOGIA: TV a schermo piatto, Canali satellitari, | SERVIZI DI RISTORAZIONE: Frutta
+a pagamento, Vino/champagne
+a pagamento, Buffet per bambini, Pasti per bambini, Menù per diete particolari (su richiesta), Snack bar, Bar, Ristorante, | INTERNET: | PARCHEGGIO: Parcheggio in strada, | ALTRI SERVIZI: Servizio navetta, Sala comune/zona TV, Servizio navetta (gratuito), Possibilità di pranzo al sacco, Servizio lavanderia
+a pagamento, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Cancelletti di sicurezza per bambini, Area giochi all'aperto, | PROTEZIONE E SICUREZZA: Estintori, Telecamere a circuito chiuso nelle zone in comune, Accesso con chiavi, | SERVIZI GENERALI: Minimarket sul posto, Aria condizionata, Struttura interamente non fumatori, Zanzariera, Riscaldamento, Ingresso indipendente, Disponibilità di camere familiari, Camere non fumatori, | 2 PISCINE: Stagionale, Recinto attorno alla piscina, Sdraio/lettini, Zona acqua bassa, Anche per bambini, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | LINGUE PARLATE: Inglese, Francese, Italiano, | </t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/villaggio-camping-blu.it.html</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>villaggio-camping-blu</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Tobacco Road camping Sirolo</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Via Peschiera 9, 60020 Sirolo, Italia</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Questa struttura si trova a 18 minuti a piedi dalla spiaggia. Situato a Sirolo, il Tobacco Road camping Sirolo offre una vista sulla sua piscina, un bar, un salotto in comune e sistemazioni con WiFi gratuito.
 Le unità dispongono di patio, cucina con frigorifero, zona pranzo, area soggiorno con TV a schermo piatto e bagno privato con doccia.
@@ -1163,12 +1215,12 @@
 I famosi luoghi di interesse nelle vicinanze del Tobacco Road camping Sirolo includono le spiagge di Urbani, San Michele e Numana. L’Aeroporto di Ancona-Falconara, il più vicino, sorge a 23 km.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>No camping host description</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t xml:space="preserve">BAGNO: Vasca o doccia, Bagno privato, WC, Doccia, | VISTA: Vista piscina, | SPAZI ALL'APERTO: Area picnic, Zona pranzo all'aperto, Barbecue, Patio, | CUCINA: Tavolo da pranzo, Utensili da cucina, Cucina, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Divano letto, Stendibiancheria, Stand appendiabiti, | ATTIVITÀ: Trasmissione di eventi sportivi in diretta, Spettacolo/musica dal vivo
 Non sul posto, Happy hour
@@ -1180,61 +1232,14 @@
 a pagamento, | ALTRI SERVIZI: Sala comune/zona TV, Check-in e check-out privati, Possibilità di pranzo al sacco, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, | PROTEZIONE E SICUREZZA: Estintori, Telecamere a circuito chiuso all'esterno della struttura, Telecamere a circuito chiuso nelle zone in comune, Accesso con chiavi, Sicurezza 24 ore su 24, | SERVIZI GENERALI: Aria condizionata, Struttura interamente non fumatori, Riscaldamento, Insonorizzazione, Ingresso indipendente, Camere non fumatori, | PISCINA SCOPERTA: Stagionale, Orari di apertura, Accessibile a ogni età, Recinto attorno alla piscina, Sdraio/lettini, Bar a bordo piscina, Zona acqua bassa, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | LINGUE PARLATE: Tedesco, Inglese, Italiano, | </t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>https://www.booking.com/hotel/it/tobacco-road.it.html</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>tobacco-road</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Safaritent Glamping Mar Y Sierrra</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>via S. Gervasio, 61039 Casa Castellani, Italia</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Situato a Casa Castellani, il Safaritent Glamping Mar Y Sierrra offre un ristorante, una piscina stagionale all'aperto e un bar. La struttura dista 37 km da Urbino e dispone di un parcheggio privato gratuito.
-In loco troverete anche un'area giochi per bambini. Durante il vostro soggiorno al Safaritent Glamping Mar Y Sierrra potrete giocare a ping pong in loco o esplorare i dintorni in bicicletta.
-La struttura dista 41 km da Ancona e 27 km da Pesaro. Il Safaritent Glamping Mar Y Sierrra dista 25 km dall'Aeroporto di Ancona Falconara, lo scalo più vicino.</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>No camping host description</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARCHEGGIO: Parcheggio per disabili, | INTERNET: | CUCINA: Utensili da cucina, | CAMERA DA LETTO: Biancheria per la casa, | BAGNO: Vasca o doccia, Bagno privato, WC, Doccia, | SPAZI ALL'APERTO: Arredamento da esterni, Arredamento da esterno, Terrazza solarium, Barbecue, Barbecue, Terrazza, Giardino, | PISCINA SCOPERTA: Stagionale, Accessibile a ogni età, Sdraio/lettini, Bar a bordo piscina, Ombrelloni, Scivolo d'acqua, Zona acqua bassa, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, Scivolo d'acqua, | SERVIZI GENERALI: Minimarket sul posto, Struttura interamente non fumatori, Zanzariera, Parquet o pavimento in legno, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Vino/champagne
-a pagamento, Pasti per bambini, Bar, Ristorante, Bollitore tè/macchina caffè, | ATTIVITÀ: Tour in bicicletta, Tour a piedi, Snorkeling
-Non sul posto, Equitazione
-Non sul posto, Escursioni in bicicletta
-Non sul posto, Vasca idromassaggio/jacuzzi, Windsurf
-Non sul posto, Ping-pong, Area giochi, Campo da tennis, | ALTRI SERVIZI: Check-in e check-out privati, | VISTA: Vista montagna, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, | LINGUE PARLATE: Tedesco, Inglese, Italiano, Olandese, | </t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/safaritent-glamping-mar-y-sierrra.it.html</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>safaritent-glamping-mar-y-sierrra</t>
         </is>
       </c>
     </row>
@@ -1244,15 +1249,59 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>Camping Liana</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lungomare Leonardo da Vinci 54 ter, 60019 Senigallia, Italia</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Situato a Senigallia, a 26 km da Ancona, il Camping Liana offre un ristorante e la connessione WiFi gratuita.
+La sistemazione dispone di aria condizionata, TV a schermo piatto, cucina interamente attrezzata con zona pranzo e bagno privato completo di doccia. Potrete usufruire di lenzuola e asciugamani a costo aggiuntivo.
+Presso il campeggio potrete gustare al mattino una colazione all’italiana.
+Il Camping Liana dista 35 km da Sirolo e 44 km da Porto Recanati. L’Aeroporto di Ancona-Falconara, lo scalo più vicino, sorge a 27 km.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No camping host description</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAGNO: Carta igienica, Asciugamani, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | VISTA: Vista luogo di interesse, Vista mare, | SPAZI ALL'APERTO: Zona pranzo all'aperto, Arredamento da esterno, Barbecue, | CUCINA: Seggiolone, Tavolo da pranzo, Piano cottura, Utensili da cucina, Cucina, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Stendibiancheria, Stand appendiabiti, | ANIMALI: | ATTIVITÀ: Spiaggia, Fronte spiaggia, Spiaggia privata
+a pagamento, | AREA SOGGIORNO: Zona pranzo, | MEDIA E TECNOLOGIA: TV a schermo piatto, TV, | SERVIZI DI RISTORAZIONE: Snack bar, Bar, Ristorante, | INTERNET: | PARCHEGGIO: | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Giochi da tavolo/puzzle, | SERVIZI GENERALI: Aria condizionata, Struttura interamente non fumatori, Zanzariera, Ingresso indipendente, Disponibilità di camere familiari, Camere non fumatori, | ACCESSIBILITÀ: Intera unità situata al piano terra, | LINGUE PARLATE: Inglese, Italiano, | </t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/camping-liana.it.html</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>camping-liana</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>Camping Norina</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Via Marina Ardizia 181, 61122 Pesaro, Italia</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Ubicato a Pesaro, il Camping Norina vanta un ristorante, un centro fitness e una spiaggia privata, e offre la connessione WiFi gratuita in tutte le aree.
 Tutti gli alloggi sono climatizzati e dotati di TV a schermo piatto e di bagno privato con asciugacapelli.
@@ -1260,42 +1309,85 @@
 La struttura dista 10 minuti di auto da Pesaro e da Fano e 23 km da Cattolica.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>No camping host description</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t xml:space="preserve">BAGNO: Asciugamani/lenzuola disponibili a pagamento, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Armadio o guardaroba, | SPAZI ALL'APERTO: Zona pranzo all'aperto, Arredamento da esterno, | CUCINA: Tavolo da pranzo, Piano cottura, Utensili da cucina, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ANIMALI: | ATTIVITÀ: Spiaggia, Fronte spiaggia, Attrezzature per sport acquatici sul posto, Spiaggia privata, Area giochi, | AREA SOGGIORNO: Zona pranzo, Divano, Zona soggiorno, | MEDIA E TECNOLOGIA: TV a schermo piatto, TV, | SERVIZI DI RISTORAZIONE: Bar, Ristorante, | INTERNET: | PARCHEGGIO: | SERVIZI GENERALI: Minimarket sul posto, Aria condizionata, Zanzariera, Riscaldamento, Ingresso indipendente, Disponibilità di camere familiari, Camere non fumatori, | LINGUE PARLATE: Tedesco, Inglese, Francese, Italiano, | </t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>https://www.booking.com/hotel/it/camping-norina.it.html</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>camping-norina</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Camping Pineta</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Via ca' mignone 5, 61029 Urbino, Italia</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Situato a Urbino, il Camping Pineta offre piscina, ristorante, bar, vista città e WiFi gratuito.
+Le sistemazioni comprendono patio, cucina con frigorifero, zona pranzo, salotto con TV e bagno privato con bidè e asciugacapelli. Per maggiore comodità, potrete usufruire di asciugamani e lenzuola ad un costo aggiuntivo.
+In loco avrete a disposizione una terrazza.
+Il Camping Pineta dista 5 km dal Duomo. L’Aeroporto Internazionale Federico Fellini è lo scalo più vicino, a 57 km dalla struttura.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ll Camping “Pineta” di Urbino è sorto in un'area di circa 22.000 metri quadri a est della citta, situato in una posizione eccellente sia dal punto di vista paesaggistico che da quello funzionale. Infatti si tratta di un terreno in declivio verso la città dal quale si gode un'ottima vista del Centro Storico. ll terreno dove sorge il Camping e in gran parte coperto da una folta pineta dando al campeggiatore uno stretto rapporto con Ia natura e il paesaggio circostante.  I servizi interni del Camping comprendono: bagni, lavandini, Iavelli, lavatoi, docce calde e fredde, fontane e torrette a norme CEE per prese di corrente (220 WT) dislocate in vari punti del terreno, tutto nelle proporzioni previste dalla legge; inoltre funzionano un Bar, un ristorante , piscina e sono disponibili anche bungalow .</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | CUCINA: Seggiolone, Tavolo da pranzo, Piano cottura, Utensili da cucina, Cucina, Frigorifero, Angolo cottura, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | BAGNO: Carta igienica, Asciugamani, Bidet, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Asciugacapelli, Doccia, | AREA SOGGIORNO: Zona pranzo, Divano, Zona soggiorno, | MEDIA E TECNOLOGIA: TV, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Divano letto, Stendibiancheria, Letto pieghevole, Stand appendiabiti, | ANIMALI: | SPAZI ALL'APERTO: Zona pranzo all'aperto, Arredamento da esterno, Terrazza solarium, Patio, Terrazza, | PISCINA SCOPERTA: Stagionale, Recinto attorno alla piscina, Piscina con vista, Zona acqua bassa, | SERVIZI BENESSERE: | SERVIZI GENERALI: Soluzioni anallergiche, Aria condizionata, Zanzariera, Parquet o pavimento in legno, Riscaldamento, Insonorizzazione, Ingresso indipendente, Disponibilità di camere familiari, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Bar, | ATTIVITÀ: Solarium, | VISTA: Vista luogo di interesse, | LINGUE PARLATE: Tedesco, Inglese, Francese, Italiano, | </t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/camping-pineta-urbino.it.html</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>camping-pineta-urbino</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Camping Paradiso</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Via Rive Del Faro 2, 61121 Pesaro, Italia</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Questa struttura si trova a 12 minuti a piedi dalla spiaggia. Ubicato nel parco regionale di San Bartolo, a 850 metri da Castel di Mezzo, il Camping Paradiso offre una piscina all'aperto e un barbecue.
 I bungalow e gli chalet dispongono di una terrazza con vista sulle montagne, di un'area salotto e, in alcuni casi, di un'angolo cottura e di una TV a schermo piatto.
@@ -1303,87 +1395,107 @@
 Il Camping Paradiso si trova a 12 km da Pesaro, e in auto dista 15 minuti dalla stazione di Cattolica e 25 minuti da Riccione.</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>La nostra peculiarità è l'atmosfera familiare unita a servizi di qualità. Da sempre i nostri ospiti possono contare sul nostro aiuto per risolvere ogni problematica ed esigenza. Non è raro trovarsi la sera insieme al bar o ristorante a scambiarci battute come amici di vecchia data. Spesso i rapporti continuano anche dopo le vacanze e le famiglie tornano a trovarci per più anni.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t xml:space="preserve">BAGNO: Carta igienica, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | SPAZI ALL'APERTO: Zona pranzo all'aperto, Arredamento da esterno, Terrazza solarium, Barbecue, Patio, Terrazza, Giardino, | CUCINA: Tavolo da pranzo, Prodotti per le pulizie, Piano cottura, Utensili da cucina, Cucina, Frigorifero, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Stendibiancheria, | ATTIVITÀ: Vasca all'aperto, Escursioni in bicicletta, Escursionismo, Freccette, Ping-pong, Area giochi, Pesca
 a pagamento, Campo da golf (nel raggio di 3 km)
 a pagamento, | AREA SOGGIORNO: Zona pranzo, Divano, Zona soggiorno, | SERVIZI DI RISTORAZIONE: Snack bar, Bar, Ristorante, | INTERNET: | PARCHEGGIO: | ALTRI SERVIZI: Sala comune/zona TV, Deposito bagagli, Fax/fotocopiatrice, Possibilità di pranzo al sacco, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, Giochi da tavolo/puzzle, | PROTEZIONE E SICUREZZA: Telecamere a circuito chiuso nelle zone in comune, Cassaforte, | SERVIZI GENERALI: Minimarket sul posto, Ingresso indipendente, Disponibilità di camere familiari, Camere non fumatori, | PISCINA SCOPERTA: Stagionale, Recinto attorno alla piscina, Sdraio/lettini, Piscina con vista, Piscina di acqua salata, Zona acqua bassa, | SERVIZI BENESSERE: Ombrelloni, Sdraio/lettini, | LINGUE PARLATE: Tedesco, Inglese, Italiano, | </t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>https://www.booking.com/hotel/it/camping-paradiso.it.html</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>camping-paradiso</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Camping Pineta</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Via ca' mignone 5, 61029 Urbino, Italia</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Situato a Urbino, il Camping Pineta offre piscina, ristorante, bar, vista città e WiFi gratuito.
-Le sistemazioni comprendono patio, cucina con frigorifero, zona pranzo, salotto con TV e bagno privato con bidè e asciugacapelli. Per maggiore comodità, potrete usufruire di asciugamani e lenzuola ad un costo aggiuntivo.
-In loco avrete a disposizione una terrazza.
-Il Camping Pineta dista 5 km dal Duomo. L’Aeroporto Internazionale Federico Fellini è lo scalo più vicino, a 57 km dalla struttura.</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>ll Camping “Pineta” di Urbino è sorto in un'area di circa 22.000 metri quadri a est della citta, situato in una posizione eccellente sia dal punto di vista paesaggistico che da quello funzionale. Infatti si tratta di un terreno in declivio verso la città dal quale si gode un'ottima vista del Centro Storico. ll terreno dove sorge il Camping e in gran parte coperto da una folta pineta dando al campeggiatore uno stretto rapporto con Ia natura e il paesaggio circostante.  I servizi interni del Camping comprendono: bagni, lavandini, Iavelli, lavatoi, docce calde e fredde, fontane e torrette a norme CEE per prese di corrente (220 WT) dislocate in vari punti del terreno, tutto nelle proporzioni previste dalla legge; inoltre funzionano un Bar, un ristorante , piscina e sono disponibili anche bungalow .</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | CUCINA: Seggiolone, Tavolo da pranzo, Piano cottura, Utensili da cucina, Cucina, Frigorifero, Angolo cottura, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | BAGNO: Carta igienica, Asciugamani, Bidet, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Asciugacapelli, Doccia, | AREA SOGGIORNO: Zona pranzo, Divano, Zona soggiorno, | MEDIA E TECNOLOGIA: TV, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Divano letto, Stendibiancheria, Letto pieghevole, Stand appendiabiti, | ANIMALI: | SPAZI ALL'APERTO: Zona pranzo all'aperto, Arredamento da esterno, Terrazza solarium, Patio, Terrazza, | PISCINA SCOPERTA: Stagionale, Recinto attorno alla piscina, Piscina con vista, Zona acqua bassa, | SERVIZI BENESSERE: | SERVIZI GENERALI: Soluzioni anallergiche, Aria condizionata, Zanzariera, Parquet o pavimento in legno, Riscaldamento, Insonorizzazione, Ingresso indipendente, Disponibilità di camere familiari, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Bar, | ATTIVITÀ: Solarium, | VISTA: Vista luogo di interesse, | LINGUE PARLATE: Tedesco, Inglese, Francese, Italiano, | </t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-pineta-urbino.it.html</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>camping-pineta-urbino</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CIVETTUOLA</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>20 Via Consolazione, 60010 Castel Colonna, Italia</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CIVETTUOLA is situated in Castel Colonna and offers a bar and a terrace. The property is 8 km from Senigallia and free private parking is available.
+Towels and bed linen are provided.
+Guests at the tented camp can enjoy a continental breakfast.
+Guests can swim in the outdoor swimming pool, go hiking or cycling, or relax in the garden and use the barbecue facilities.
+Sirolo is 43 km from CIVETTUOLA, while Ancona is 32 km from the property. The nearest airport is Ancona Falconara Airport, 20 km from the accommodation.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Piccola tenda fissa posizionata nel bordo del parco della struttura principale. Intima, esclusiva, panoramica.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | CUCINA: Prodotti per le pulizie, Utensili da cucina, Lavatrice, Frigorifero, | CAMERA DA LETTO: Biancheria per la casa, | BAGNO: Carta igienica, Asciugamani, Servizi igienici in comune, Bagno privato, Doccia, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, | ANIMALI: | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Zona pranzo all'aperto, Arredamento da esterno, Barbecue, Barbecue, Patio, Balcone, Terrazza, Giardino, | PISCINA SCOPERTA: Stagionale, Accessibile a ogni età, Sdraio/lettini, Giochi da piscina, Piscina con vista, Zona acqua bassa, | SERVIZI BENESSERE: Sdraio/lettini, | SERVIZI GENERALI: Ciotole per animali domestici, Ceste per animali domestici, Area fumatori, Ingresso indipendente, Possibilità di pranzo al sacco, Navetta aeroportuale, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Caffetteria sul posto, Frutta
+a pagamento, Vino/champagne
+a pagamento, Bar, | ATTIVITÀ: Tiro con l'arco, Tour o lezioni sulla cultura locale, Happy hour
+a pagamento, Tour in bicicletta, Tour a piedi, Massaggi corpo
+a pagamento, Massaggi mani
+a pagamento, Massaggi testa
+a pagamento, Massaggi di coppia
+a pagamento, Massaggi piedi
+a pagamento, Massaggi collo
+a pagamento, Massaggi schiena
+a pagamento, Equitazione
+Non sul posto
+a pagamento, Escursioni in bicicletta
+Non sul posto, Escursionismo
+Non sul posto, Massaggi
+a pagamento, Pesca
+Non sul posto, | VISTA: Vista luogo di interesse, Vista giardino, | TRASPORTI: Navetta per l'aeroporto
+a pagamento, Navetta dall'aeroporto
+a pagamento, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, Check-in e check-out privati, Deposito bagagli, Check-in e check-out express, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, | SERVIZI BUSINESS: Fax/fotocopiatrice
+a pagamento, | PROTEZIONE E SICUREZZA: Accesso con chiavi, Sicurezza 24 ore su 24, | LINGUE PARLATE: Inglese, Spagnolo, Italiano, | </t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/hotel/it/civettuola.it.html</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>civettuola</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>Camping Village Costa Verde</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Contrada Asola, 62018 Porto Potenza Picena, Italia</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Questa struttura si trova a 3 minuti a piedi dalla spiaggia. Situato a Porto Potenza Picena, a 200 metri dalle spiagge di sabbia, il Camping Village Costa Verde offre una piscina all'aperto, un ristorante e la connessione Wi-Fi gratuita nelle aree comuni.
 La struttura metterà a vostra disposizione una reception aperta 24 ore su 24, programmi di intrattenimento serali e per bambini, un'area TV in comune e alcuni servizi a pagamento, come il noleggio di biciclette o di sedie a sdraio per la spiaggia privata.
@@ -1392,12 +1504,12 @@
 Dotato di parcheggio gratuito, il campeggio dista 11,5 km da Porto Sant'Elpidio e 20 minuti di auto dal punto di inizio del Parco Regionale del Conero.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Il Camping Village Costa Verde si trova nelle Marche, a pochi chilometri da una delle aree più suggestive della splendida riviera Adriatica, il Parco naturale del Conero.</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t xml:space="preserve">BAGNO: Asciugamani/lenzuola disponibili a pagamento, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Armadio o guardaroba, | SPAZI ALL'APERTO: Zona pranzo all'aperto, Arredamento da esterno, Barbecue, | CUCINA: Seggiolone, Tavolo da pranzo, Prodotti per le pulizie, Piano cottura, Utensili da cucina, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Stendibiancheria, Stand appendiabiti, | ANIMALI: | ATTIVITÀ: Spiaggia, Intrattenimento serale, Attrezzature per sport acquatici sul posto
 a pagamento, Staff di animazione, Spiaggia privata
@@ -1409,107 +1521,14 @@
 a pagamento, Riscaldamento, Disponibilità di camere familiari, | LINGUE PARLATE: Inglese, Italiano, | </t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>https://www.booking.com/hotel/it/camping-village-costa-verde.it.html</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>camping-village-costa-verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Camping Liana</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Lungomare Leonardo da Vinci 54 ter, 60019 Senigallia, Italia</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Situato a Senigallia, a 26 km da Ancona, il Camping Liana offre un ristorante e la connessione WiFi gratuita.
-La sistemazione dispone di aria condizionata, TV a schermo piatto, cucina interamente attrezzata con zona pranzo e bagno privato completo di doccia. Potrete usufruire di lenzuola e asciugamani a costo aggiuntivo.
-Presso il campeggio potrete gustare al mattino una colazione all’italiana.
-Il Camping Liana dista 35 km da Sirolo e 44 km da Porto Recanati. L’Aeroporto di Ancona-Falconara, lo scalo più vicino, sorge a 27 km.</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>No camping host description</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BAGNO: Carta igienica, Asciugamani, Asciugamani/lenzuola disponibili a pagamento, Vasca o doccia, Bagno privato, WC, Doccia, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | VISTA: Vista luogo di interesse, Vista mare, | SPAZI ALL'APERTO: Zona pranzo all'aperto, Arredamento da esterno, Barbecue, | CUCINA: Seggiolone, Tavolo da pranzo, Piano cottura, Utensili da cucina, Cucina, Frigorifero, Angolo cottura, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Stendibiancheria, Stand appendiabiti, | ANIMALI: | ATTIVITÀ: Spiaggia, Fronte spiaggia, Spiaggia privata
-a pagamento, | AREA SOGGIORNO: Zona pranzo, | MEDIA E TECNOLOGIA: TV a schermo piatto, TV, | SERVIZI DI RISTORAZIONE: Snack bar, Bar, Ristorante, | INTERNET: | PARCHEGGIO: | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Giochi da tavolo/puzzle, | SERVIZI GENERALI: Aria condizionata, Struttura interamente non fumatori, Zanzariera, Ingresso indipendente, Disponibilità di camere familiari, Camere non fumatori, | ACCESSIBILITÀ: Intera unità situata al piano terra, | LINGUE PARLATE: Inglese, Italiano, | </t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-liana.it.html</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>camping-liana</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>fattoria country village</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>contrada fonte san giovanni 3 montecarotto contrada fonte san giovanni 3, 60036 Montecarotto, Italia</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Hai diritto a uno sconto Genius su fattoria country village! Per risparmiare su questa struttura ti basta accedere.
-Situato a Montecarotto, nelle Marche, il Fattoria Country Village offre sistemazioni con parcheggio privato gratuito.
-A disposizione un bagno in comune completamente attrezzato con bidet e set di cortesia.
-Al mattino vi attende una colazione a buffet o all'italiana.
-Potrete approfittare di un barbecue e rilassarvi in giardino o nell’area salotto in comune.
-Il Fattoria Country Village dista 45 km da Sirolo e 26 km da Senigallia. A 39 km raggiungerete l’Aeroporto di Ancona-Falconara, lo scalo più vicino.</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>No camping host description</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARCHEGGIO: Parcheggio custodito, | INTERNET: | CUCINA: Cucina in comune, | BAGNO: Carta igienica, Bidet, Vasca o doccia, Servizi igienici in comune, WC, Prodotti da bagno in omaggio, Bagno in comune, Vasca, Doccia, | AREA SOGGIORNO: Zona soggiorno, | SERVIZI IN CAMERA: Stendibiancheria, | ANIMALI: | ACCESSIBILITÀ: Campanello di emergenza nel bagno, Lavabo più basso, WC con seduta più alta, WC con maniglioni, Accesso su sedia a rotelle, | SPAZI ALL'APERTO: Camino all'aperto, Area picnic, Barbecue, Barbecue, Giardino, | PISCINA SCOPERTA: Stagionale, Orari di apertura, Accessibile a ogni età, Teli da piscina/spiaggia, Sdraio/lettini, Giochi da piscina, Ombrelloni, Piscina con vista, | SERVIZI BENESSERE: Sdraio/lettini, Teli da piscina/spiaggia, | SERVIZI GENERALI: Ciotole per animali domestici, WiFi a pagamento, Sala comune/zona TV, Servizio navetta (a pagamento), Possibilità di pranzo al sacco, Cappella o luogo di culto, Camere/strutture per ospiti disabili, Cassaforte, | SERVIZI DI RISTORAZIONE: Caffetteria sul posto, Vino/champagne
-a pagamento, Pasti per bambini, Snack bar, | ATTIVITÀ: Tiro con l'arco, Happy hour
-a pagamento, Tour in bicicletta, Tour a piedi
-a pagamento, Giro dei pub
-a pagamento, Attrezzatura da badminton, Vasca all'aperto, Staff di animazione, Escursioni in bicicletta, Ping-pong, Pesca, | VISTA: Vista, | SERVIZI DI ACCOGLIENZA: Check-in e check-out privati, Reception 24 ore su 24, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Area giochi all'aperto, Area giochi al coperto, Giochi da tavolo/puzzle, | SERVIZI BUSINESS: Fax/fotocopiatrice, | LINGUE PARLATE: Inglese, Spagnolo, | </t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/fattoria-country-village.it.html</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>fattoria-country-village</t>
         </is>
       </c>
     </row>
@@ -1519,46 +1538,43 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bungalow Verde Mare</t>
+          <t>Glamping Marche Nascoste Tenda e intero alloggio</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Lungomare Marina Palmense, 63900 Marina Palmense, Italia</t>
+          <t>41 Strada Provinciale 54, 62020 Penna San Giovanni, Italia</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Offering sea views and a seasonal outdoor swimming pool, Bungalow Verde Mare offers accommodation conveniently located in Marina Palmense, within a short distance of Porto San Giorgio Beach.
-The camping offers a seating area with a flat-screen TV and a private bathroom with a hairdryer and bidet.
-A children's playground is also available for guests at Bungalow Verde Mare.
-The nearest airport is Ancona Falconara Airport, 62 km from the accommodation.</t>
+          <t>Located in Penna San Giovanni in the Marche region, Glamping Marche Nascoste Tenda e intero alloggio features a garden. The property is 39 km from Grottammare and free private parking is provided.
+The tented camp also provides a fully equipped kitchen with a fridge, a seating area, a washing machine and 1 bathroom with a bidet and a bath.
+An Italian breakfast is available daily at the tented camp.
+San Benedetto del Tronto is 41 km from Glamping Marche Nascoste Tenda, while Porto Recanati is 47 km away. The nearest airport is Ancona Falconara Airport, 61 km from the accommodation.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>No camping host description</t>
+          <t>Nel piccolo borgo di Penna San Giovanni potrete soggiornare nella tenda Sibilla ,all'ombra degli alberi del nostro giardino con vista sui Sibillini, tra ulivi e fiori. Tenda di 5 m di diametro arredata (max 4 pers.) e intero alloggio privato con bagno, cucina, una camera (altre 2 pers.), sala e intrattenimento per vivere momenti meravigliosi. L'alloggio può ospitare fino a 6 persone dello stesso nucleo.
+Colazione con prodotti freschi locali. Noleggio bici, trekking, spiagge nelle vicinanze e molto altro!
+La nostra filosofia: green, fai da te, riutilizzo per limitare l'impatto ambientale.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAGNO: Carta igienica, Bidet, Bagno privato, WC, Asciugacapelli, | VISTA: Vista mare, | SPAZI ALL'APERTO: Zona pranzo all'aperto, Arredamento da esterno, Barbecue, | CUCINA: Tavolo da pranzo, Piano cottura, Utensili da cucina, Lavatrice, Frigorifero, | SERVIZI IN CAMERA: Divano letto, Stendibiancheria, Stand appendiabiti, | ANIMALI: | ATTIVITÀ: Happy hour
-a pagamento, Spiaggia, Attrezzatura da tennis
-a pagamento, Intrattenimento serale, Locale notturno/DJ, Staff di animazione, Area giochi, Campo da tennis
-a pagamento, | AREA SOGGIORNO: Zona pranzo, Divano, Zona soggiorno, | MEDIA E TECNOLOGIA: TV a schermo piatto, | INTERNET: | PARCHEGGIO: | ALTRI SERVIZI: Servizio lavanderia
-a pagamento, Servizio baby-sitter
-a pagamento, | SERVIZI GENERALI: Minimarket sul posto, Ferro e asse da stiro, | PISCINA SCOPERTA: Stagionale, Accessibile a ogni età, Sdraio/lettini, Bar a bordo piscina, Ombrelloni, Scivolo d'acqua, | SERVIZI BENESSERE: Ombrelloni
-a pagamento, Sdraio/lettini, Scivolo d'acqua, | LINGUE PARLATE: Inglese, Italiano, | </t>
+          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | CUCINA: Tavolo da pranzo, Prodotti per le pulizie, Tostapane, Piano cottura, Forno, Utensili da cucina, Cucina, Lavatrice, Frigorifero, Angolo cottura, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | BAGNO: Asciugamani, Bidet, Vasca o doccia, Servizi igienici in comune, Bagno privato, WC, Prodotti da bagno in omaggio, Asciugacapelli, Vasca, | AREA SOGGIORNO: Zona pranzo, Divano, Zona soggiorno, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Stendibiancheria, Stand appendiabiti, | ANIMALI: | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Zona pranzo all'aperto, Arredamento da esterno, Barbecue, Barbecue, Giardino, | SERVIZI GENERALI: Zanzariera, Pavimento in marmo o in piastrelle, Ingresso indipendente, Riscaldamento, Ventilatore, Disponibilità di camere familiari, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Frutta, Vino/champagne
+a pagamento, Possibilità di colazione in camera, Bollitore tè/macchina caffè, | ATTIVITÀ: Freccette, Ping-pong, | ALTRI SERVIZI: Ciotole per animali domestici, Servizio lavanderia, | VISTA: Vista montagna, Vista giardino, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Giochi da tavolo/puzzle, Giochi da tavolo/puzzle, | LINGUE PARLATE: Tedesco, Inglese, Spagnolo, Italiano, | </t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/bungalow-verde-mare.it.html</t>
+          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>bungalow-verde-mare</t>
+          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
         </is>
       </c>
     </row>
@@ -1616,43 +1632,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Glamping Marche Nascoste Tenda e intero alloggio</t>
+          <t>Camping Villaggio Cortina</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>41 Strada Provinciale 54, 62020 Penna San Giovanni, Italia</t>
+          <t>Lungomare Italia 1/1, 60019 Senigallia, Italia</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Located in Penna San Giovanni in the Marche region, Glamping Marche Nascoste Tenda e intero alloggio features a garden. The property is 39 km from Grottammare and free private parking is provided.
-The tented camp also provides a fully equipped kitchen with a fridge, a seating area, a washing machine and 1 bathroom with a bidet and a bath.
-An Italian breakfast is available daily at the tented camp.
-San Benedetto del Tronto is 41 km from Glamping Marche Nascoste Tenda, while Porto Recanati is 47 km away. The nearest airport is Ancona Falconara Airport, 61 km from the accommodation.</t>
+          <t>Questa struttura si trova a 1 minuto a piedi dalla spiaggia. Il Camping Villaggio Cortina sorge sul lungomare di Senigallia, proprio di fronte alla spiaggia. Offre la connessione Wi-Fi gratuita nella zona della reception.
+Alcune unità sono dotate di aria condizionata, angolo cottura con frigorifero e zona pranzo.
+La struttura dispone di un bar in loco dove potrete gustare un drink. A vostra disposizione anche una spiaggia privata.
+Il Camping Cortina dista 5 km dalla stazione ferroviaria di Senigallia e 24 km da Ancona.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Nel piccolo borgo di Penna San Giovanni potrete soggiornare nella tenda Sibilla ,all'ombra degli alberi del nostro giardino con vista sui Sibillini, tra ulivi e fiori. Tenda di 5 m di diametro arredata (max 4 pers.) e intero alloggio privato con bagno, cucina, una camera (altre 2 pers.), sala e intrattenimento per vivere momenti meravigliosi. L'alloggio può ospitare fino a 6 persone dello stesso nucleo.
-Colazione con prodotti freschi locali. Noleggio bici, trekking, spiagge nelle vicinanze e molto altro!
-La nostra filosofia: green, fai da te, riutilizzo per limitare l'impatto ambientale.</t>
+          <t>Da più di 15 anni ospitiamo famiglie, coppie e campeggiatori nella nostra struttura. 
+Abbiamo piazzole per tende, roulotte e camper e comode mobilhouse da 4 o 5 posti.
+Il nostro pacchetto all-inclusive vi permette di pagare una sola volta per avere tutto ciò che può servirvi, mobilhouse, parcheggio, pulizie animazione e servizio spiaggia tutto compreso!
+Voi dovrete portare soltando la crema solare!</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARCHEGGIO: | INTERNET: | CUCINA: Tavolo da pranzo, Prodotti per le pulizie, Tostapane, Piano cottura, Forno, Utensili da cucina, Cucina, Lavatrice, Frigorifero, Angolo cottura, | CAMERA DA LETTO: Biancheria per la casa, Armadio o guardaroba, | BAGNO: Asciugamani, Bidet, Vasca o doccia, Servizi igienici in comune, Bagno privato, WC, Prodotti da bagno in omaggio, Asciugacapelli, Vasca, | AREA SOGGIORNO: Zona pranzo, Divano, Zona soggiorno, | SERVIZI IN CAMERA: Presa elettrica vicino al letto, Stendibiancheria, Stand appendiabiti, | ANIMALI: | SPAZI ALL'APERTO: Area picnic, Arredamento da esterni, Zona pranzo all'aperto, Arredamento da esterno, Barbecue, Barbecue, Giardino, | SERVIZI GENERALI: Zanzariera, Pavimento in marmo o in piastrelle, Ingresso indipendente, Riscaldamento, Ventilatore, Disponibilità di camere familiari, Camere non fumatori, | SERVIZI DI RISTORAZIONE: Frutta, Vino/champagne
-a pagamento, Possibilità di colazione in camera, Bollitore tè/macchina caffè, | ATTIVITÀ: Freccette, Ping-pong, | ALTRI SERVIZI: Ciotole per animali domestici, Servizio lavanderia, | VISTA: Vista montagna, Vista giardino, | INTRATTENIMENTO E SERVIZI PER LE FAMIGLIE: Giochi da tavolo/puzzle, Giochi da tavolo/puzzle, | LINGUE PARLATE: Tedesco, Inglese, Spagnolo, Italiano, | </t>
+          <t xml:space="preserve">BAGNO: Asciugamani/lenzuola disponibili a pagamento, | SPAZI ALL'APERTO: Arredamento da esterni, Barbecue, Terrazza, Giardino, | CUCINA: Frigorifero, | SERVIZI IN CAMERA: Stendibiancheria, | ANIMALI: | ATTIVITÀ: Spiaggia, Intrattenimento serale, Fronte spiaggia, Staff di animazione, Spiaggia privata, Windsurf
+Non sul posto
+a pagamento, Ping-pong, | SERVIZI DI RISTORAZIONE: Pasti per bambini
+a pagamento, Snack bar, Bar, Ristorante, | INTERNET: | PARCHEGGIO: Parcheggio per disabili, Parcheggio in strada, | TRASPORTI: Biglietti per i mezzi di trasporto, | ALTRI SERVIZI: Servizio navetta, Servizio lavanderia
+a pagamento, | SERVIZI DI ACCOGLIENZA: Fattura disponibile su richiesta, | PROTEZIONE E SICUREZZA: Estintori, Accesso con chiavi, | SERVIZI GENERALI: Aria condizionata, Riscaldamento, Ingresso indipendente, Disponibilità di camere familiari, Camere/strutture per ospiti disabili, Camere non fumatori, | ACCESSIBILITÀ: Lavabo più basso, WC con maniglioni, Accesso su sedia a rotelle, | SERVIZI BENESSERE: Ombrelloni, | LINGUE PARLATE: Inglese, Italiano, | </t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html</t>
+          <t>https://www.booking.com/hotel/it/villaggio-cortina.it.html</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
+          <t>villaggio-cortina</t>
         </is>
       </c>
     </row>

</xml_diff>